<commit_message>
correções de lógica de modelo excel, botões sumindo ao editar
</commit_message>
<xml_diff>
--- a/templates/FICHA DE IMÓVEL.xlsx
+++ b/templates/FICHA DE IMÓVEL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bfadada786324fd2/Documentos/Projetos/OrganizadorDocumentos/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="13_ncr:1_{D551FD33-9428-497F-8EF4-8ACFB4143F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6255E877-20DE-4656-B7B4-A6A0E671AFB6}"/>
+  <xr:revisionPtr revIDLastSave="157" documentId="13_ncr:1_{D551FD33-9428-497F-8EF4-8ACFB4143F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08439368-C2CF-4FC5-AF37-0D1D2563FC1C}"/>
   <bookViews>
-    <workbookView xWindow="-20355" yWindow="4740" windowWidth="20460" windowHeight="10770" xr2:uid="{7C6B54FE-6144-4091-84F2-B755001FC5E3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7C6B54FE-6144-4091-84F2-B755001FC5E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>FICHA DE CLIENTES</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t xml:space="preserve">NOME DO CONTRANTE </t>
+  </si>
+  <si>
+    <t>Sem detalhes</t>
   </si>
 </sst>
 </file>
@@ -117,7 +120,7 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -193,6 +196,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -346,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -359,9 +370,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="8" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -386,12 +394,75 @@
     <xf numFmtId="16" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -401,41 +472,24 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -444,24 +498,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -808,17 +844,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
@@ -834,260 +870,260 @@
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
       <c r="J3" s="6"/>
     </row>
     <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="F4" s="12" t="s">
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="F4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42"/>
       <c r="J4" s="6"/>
     </row>
     <row r="5" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="13"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="12"/>
     </row>
     <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="10" t="s">
+      <c r="B7" s="42"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
-      <c r="I7" s="22"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
       <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:10" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="17"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="26"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="20"/>
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="17"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="29"/>
+      <c r="A12" s="16"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="23"/>
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="26"/>
+      <c r="A13" s="16"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="20"/>
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A14" s="17"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
-      <c r="I14" s="32"/>
+      <c r="A14" s="16"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="26"/>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="17"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="35"/>
+      <c r="A15" s="16"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="29"/>
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="36"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="38"/>
+      <c r="A18" s="32"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="34"/>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="39"/>
-      <c r="B19" s="40"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="40"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="41"/>
+      <c r="A19" s="35"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="37"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="39"/>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="40"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="41"/>
+      <c r="A20" s="35"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="37"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="39"/>
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="41"/>
+      <c r="A21" s="35"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="37"/>
       <c r="J21" s="1"/>
     </row>
     <row r="22" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="42"/>
-      <c r="B22" s="43"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="43"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="43"/>
-      <c r="I22" s="44"/>
+      <c r="A22" s="38"/>
+      <c r="B22" s="39"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="39"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="39"/>
+      <c r="I22" s="40"/>
       <c r="J22" s="1"/>
     </row>
     <row r="24" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
+      <c r="A24" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="30"/>
     </row>
     <row r="26" spans="1:10" s="4" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
@@ -1128,17 +1164,17 @@
       <c r="J29" s="1"/>
     </row>
     <row r="30" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
+      <c r="B30" s="30"/>
+      <c r="C30" s="30"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="30"/>
       <c r="J30" s="1"/>
     </row>
     <row r="31" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
@@ -1161,7 +1197,7 @@
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
     </row>
-    <row r="33" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>6</v>
       </c>
@@ -1177,7 +1213,7 @@
       </c>
       <c r="I33" s="1"/>
     </row>
-    <row r="34" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>7</v>
       </c>
@@ -1193,101 +1229,107 @@
       </c>
       <c r="I34" s="1"/>
     </row>
-    <row r="36" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="19" t="s">
+    <row r="36" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="19"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="19"/>
-    </row>
-    <row r="37" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="36"/>
-      <c r="B37" s="37"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="37"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="37"/>
-      <c r="I37" s="38"/>
-    </row>
-    <row r="38" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="39"/>
-      <c r="B38" s="40"/>
-      <c r="C38" s="40"/>
-      <c r="D38" s="40"/>
-      <c r="E38" s="40"/>
-      <c r="F38" s="40"/>
-      <c r="G38" s="40"/>
-      <c r="H38" s="40"/>
-      <c r="I38" s="41"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="39"/>
-      <c r="B39" s="40"/>
-      <c r="C39" s="40"/>
-      <c r="D39" s="40"/>
-      <c r="E39" s="40"/>
-      <c r="F39" s="40"/>
-      <c r="G39" s="40"/>
-      <c r="H39" s="40"/>
-      <c r="I39" s="41"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="42"/>
-      <c r="B40" s="43"/>
-      <c r="C40" s="43"/>
-      <c r="D40" s="43"/>
-      <c r="E40" s="43"/>
-      <c r="F40" s="43"/>
-      <c r="G40" s="43"/>
-      <c r="H40" s="43"/>
-      <c r="I40" s="44"/>
-    </row>
-    <row r="42" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="A42" s="15" t="s">
+      <c r="B36" s="30"/>
+      <c r="C36" s="30"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="30"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="30"/>
+      <c r="I36" s="30"/>
+    </row>
+    <row r="37" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="51" t="s">
+        <v>24</v>
+      </c>
+      <c r="B37" s="52"/>
+      <c r="C37" s="52"/>
+      <c r="D37" s="52"/>
+      <c r="E37" s="52"/>
+      <c r="F37" s="52"/>
+      <c r="G37" s="52"/>
+      <c r="H37" s="52"/>
+      <c r="I37" s="53"/>
+    </row>
+    <row r="38" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="45"/>
+      <c r="B38" s="46"/>
+      <c r="C38" s="46"/>
+      <c r="D38" s="46"/>
+      <c r="E38" s="46"/>
+      <c r="F38" s="46"/>
+      <c r="G38" s="46"/>
+      <c r="H38" s="46"/>
+      <c r="I38" s="47"/>
+      <c r="J38" s="44"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="45"/>
+      <c r="B39" s="46"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="46"/>
+      <c r="E39" s="46"/>
+      <c r="F39" s="46"/>
+      <c r="G39" s="46"/>
+      <c r="H39" s="46"/>
+      <c r="I39" s="47"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="45"/>
+      <c r="B40" s="46"/>
+      <c r="C40" s="46"/>
+      <c r="D40" s="46"/>
+      <c r="E40" s="46"/>
+      <c r="F40" s="46"/>
+      <c r="G40" s="46"/>
+      <c r="H40" s="46"/>
+      <c r="I40" s="47"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="45"/>
+      <c r="B41" s="46"/>
+      <c r="C41" s="46"/>
+      <c r="D41" s="46"/>
+      <c r="E41" s="46"/>
+      <c r="F41" s="46"/>
+      <c r="G41" s="46"/>
+      <c r="H41" s="46"/>
+      <c r="I41" s="47"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="48"/>
+      <c r="B42" s="49"/>
+      <c r="C42" s="49"/>
+      <c r="D42" s="49"/>
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
+      <c r="G42" s="49"/>
+      <c r="H42" s="49"/>
+      <c r="I42" s="50"/>
+    </row>
+    <row r="44" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B42" s="15"/>
-      <c r="C42" s="20">
+      <c r="B44" s="14"/>
+      <c r="C44" s="31">
         <v>0</v>
       </c>
-      <c r="D42" s="20"/>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="20"/>
-      <c r="H42" s="20"/>
-      <c r="I42" s="20"/>
-    </row>
-    <row r="43" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="D43" s="8"/>
-      <c r="E43" s="8"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="1"/>
-      <c r="H43" s="8"/>
-      <c r="I43" s="8"/>
-    </row>
-    <row r="44" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="1"/>
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
-      <c r="G44" s="6"/>
-      <c r="H44" s="1"/>
-      <c r="I44" s="1"/>
-    </row>
-    <row r="45" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D44" s="31"/>
+      <c r="E44" s="31"/>
+      <c r="F44" s="31"/>
+      <c r="G44" s="31"/>
+      <c r="H44" s="31"/>
+      <c r="I44" s="31"/>
+    </row>
+    <row r="45" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="7"/>
-      <c r="C45" s="9"/>
+      <c r="C45" s="8"/>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
       <c r="F45" s="6"/>
@@ -1304,19 +1346,17 @@
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="B3:I3"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A17:I17"/>
     <mergeCell ref="A24:I24"/>
-    <mergeCell ref="C42:I42"/>
+    <mergeCell ref="C44:I44"/>
     <mergeCell ref="A18:I18"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="A20:I20"/>
     <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A37:I40"/>
     <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A37:I42"/>
     <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A44:B44"/>
     <mergeCell ref="A9:I9"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A12:B12"/>
@@ -1328,6 +1368,8 @@
     <mergeCell ref="C13:I13"/>
     <mergeCell ref="C14:I14"/>
     <mergeCell ref="C15:I15"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A36:I36"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>